<commit_message>
Ajustes de pantallas: Derivados sin opciones y propósito cobertura/inversión, Módulos conectados en todas, catálogos y flujo editables, filtros por tipo de activo, tarjetas balanceadas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01LasPtPWZ9DiXFQxAHJhmgi
</commit_message>
<xml_diff>
--- a/Plantillas_carga_masiva/Chile/Ejemplo_Cargue_Masivo_Ordenes_de_Renta_Fija.xlsx
+++ b/Plantillas_carga_masiva/Chile/Ejemplo_Cargue_Masivo_Ordenes_de_Renta_Fija.xlsx
@@ -306,7 +306,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="A2:A1000">
-      <formula1>Listas!$A$2:$A$20</formula1>
+      <formula1>Listas!$A$2:$A$15</formula1>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="B2:B1000">
       <formula1>Listas!$B$2:$B$3</formula1>
@@ -668,7 +668,7 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t xml:space="preserve">Julian Andres Mesa Restrepo</t>
+          <t xml:space="preserve">FONDO INMOBILIARIO 1</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
@@ -685,7 +685,7 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t xml:space="preserve">Andres Julian Murillo Lopez</t>
+          <t xml:space="preserve">FONDO ALTERNATIVO 1</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
@@ -702,7 +702,7 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t xml:space="preserve">Gustavo Saldarriaga</t>
+          <t xml:space="preserve">APV CONSERVADOR</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
@@ -719,7 +719,7 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t xml:space="preserve">Paula Andrea Alvarez</t>
+          <t xml:space="preserve">APV MODERADO</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
@@ -736,7 +736,7 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t xml:space="preserve">Grupo Corporativo Jham</t>
+          <t xml:space="preserve">APV AGRESIVO</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
@@ -747,91 +747,6 @@
       <c r="C15" t="inlineStr">
         <is>
           <t xml:space="preserve">SURA</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FONDO INMOBILIARIO 1</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t xml:space="preserve">FONDO ALTERNATIVO 1</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t xml:space="preserve">APV CONSERVADOR</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t xml:space="preserve">APV MODERADO</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t xml:space="preserve">APV AGRESIVO</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t xml:space="preserve"/>
         </is>
       </c>
     </row>

</xml_diff>